<commit_message>
Incluir urbanismo en avance ponderado
</commit_message>
<xml_diff>
--- a/tests/fixtures/cubicacion-caratula-acumulado.xlsx
+++ b/tests/fixtures/cubicacion-caratula-acumulado.xlsx
@@ -3,7 +3,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>CUBICACION Nro. 8</t>
   </si>
@@ -30,9 +30,6 @@
   </si>
   <si>
     <t>Actual Acumulado</t>
-  </si>
-  <si>
-    <t>URBANISMO</t>
   </si>
   <si>
     <t>EDIFICIO 76</t>
@@ -89,9 +86,6 @@
       <c r="A4">
         <v>1</v>
       </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
       <c r="C4">
         <v>100</v>
       </c>
@@ -119,7 +113,7 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -148,7 +142,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -172,6 +166,17 @@
         <v>0.09</v>
       </c>
     </row>
+    <row r="7">
+      <c r="C7">
+        <v>300</v>
+      </c>
+      <c r="H7">
+        <v>42</v>
+      </c>
+      <c r="I7">
+        <v>0.14</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>